<commit_message>
Đồng bộ dữ liệu Excel từ OneDrive
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30520"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phamuc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C222E481-7B79-46E3-9E53-8052F3DFC94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{C222E481-7B79-46E3-9E53-8052F3DFC94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FCC01D6-639F-431E-B1FA-AE816CFA0590}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="878" xr2:uid="{436DC667-A705-4C81-9EE1-C1CFDFA6CB8A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="878" activeTab="2" xr2:uid="{436DC667-A705-4C81-9EE1-C1CFDFA6CB8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Code màng" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="473">
   <si>
     <t>Mã màng</t>
   </si>
@@ -1021,19 +1021,16 @@
     <t>Sinomech</t>
   </si>
   <si>
-    <t>Sinomech1</t>
+    <t>Mới 1</t>
+  </si>
+  <si>
+    <t>Yoden 600</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
   <si>
     <t>Mới 2</t>
-  </si>
-  <si>
-    <t>Yoden 600</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Mới 1</t>
   </si>
   <si>
     <t>Máy</t>
@@ -3884,19 +3881,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>445</v>
+      </c>
+      <c r="B1" t="s">
         <v>446</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>447</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>448</v>
       </c>
-      <c r="D1" t="s">
-        <v>449</v>
-      </c>
       <c r="E1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -3913,7 +3910,7 @@
         <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3930,7 +3927,7 @@
         <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3947,7 +3944,7 @@
         <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -3964,7 +3961,7 @@
         <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -3981,7 +3978,7 @@
         <v>6</v>
       </c>
       <c r="E6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
   </sheetData>
@@ -4002,33 +3999,33 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1" t="s">
         <v>450</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>451</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>452</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>453</v>
-      </c>
-      <c r="E1" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C2" t="s">
         <v>455</v>
       </c>
-      <c r="B2" t="s">
-        <v>350</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>456</v>
-      </c>
-      <c r="D2" t="s">
-        <v>457</v>
       </c>
       <c r="E2">
         <v>790</v>
@@ -4036,16 +4033,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>457</v>
+      </c>
+      <c r="B3" t="s">
         <v>458</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>459</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>460</v>
-      </c>
-      <c r="D3" t="s">
-        <v>461</v>
       </c>
       <c r="E3">
         <v>790</v>
@@ -4053,16 +4050,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
+        <v>461</v>
+      </c>
+      <c r="B4" t="s">
         <v>462</v>
       </c>
-      <c r="B4" t="s">
-        <v>463</v>
-      </c>
       <c r="C4" t="s">
+        <v>459</v>
+      </c>
+      <c r="D4" t="s">
         <v>460</v>
-      </c>
-      <c r="D4" t="s">
-        <v>461</v>
       </c>
       <c r="E4">
         <v>690</v>
@@ -4070,16 +4067,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
+        <v>463</v>
+      </c>
+      <c r="B5" t="s">
         <v>464</v>
       </c>
-      <c r="B5" t="s">
-        <v>465</v>
-      </c>
       <c r="C5" t="s">
+        <v>459</v>
+      </c>
+      <c r="D5" t="s">
         <v>460</v>
-      </c>
-      <c r="D5" t="s">
-        <v>461</v>
       </c>
       <c r="E5">
         <v>590</v>
@@ -4087,16 +4084,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
+        <v>465</v>
+      </c>
+      <c r="B6" t="s">
         <v>466</v>
       </c>
-      <c r="B6" t="s">
-        <v>467</v>
-      </c>
       <c r="C6" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D6" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="E6">
         <v>950</v>
@@ -4104,16 +4101,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
+        <v>467</v>
+      </c>
+      <c r="B7" t="s">
         <v>468</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>469</v>
       </c>
-      <c r="C7" t="s">
-        <v>470</v>
-      </c>
       <c r="D7" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="E7">
         <v>950</v>
@@ -4131,18 +4128,18 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
+        <v>471</v>
+      </c>
+      <c r="B3" t="s">
         <v>472</v>
-      </c>
-      <c r="B3" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -4317,7 +4314,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3CFB6D2-CE8B-487F-94C7-1C34A36F699B}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="17.25"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -4381,11 +4378,6 @@
     <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>324</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -4417,7 +4409,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B2">
         <v>950</v>
@@ -4426,7 +4418,7 @@
         <v>790</v>
       </c>
       <c r="D2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E2">
         <v>400</v>
@@ -4434,12 +4426,12 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -4454,13 +4446,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>328</v>
+      </c>
+      <c r="B1" t="s">
         <v>329</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>330</v>
-      </c>
-      <c r="C1" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -5454,45 +5446,45 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B1" t="s">
         <v>332</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>333</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>334</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>335</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>336</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>337</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>338</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>339</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>340</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>341</v>
-      </c>
-      <c r="K1" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B2" t="s">
         <v>343</v>
-      </c>
-      <c r="B2" t="s">
-        <v>344</v>
       </c>
       <c r="D2">
         <v>150</v>
@@ -5501,24 +5493,24 @@
         <v>150</v>
       </c>
       <c r="F2" t="s">
+        <v>344</v>
+      </c>
+      <c r="G2" t="s">
         <v>345</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>346</v>
-      </c>
-      <c r="H2" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
+        <v>347</v>
+      </c>
+      <c r="B3" t="s">
         <v>348</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>349</v>
-      </c>
-      <c r="C3" t="s">
-        <v>350</v>
       </c>
       <c r="D3">
         <v>500</v>
@@ -5536,24 +5528,24 @@
         <v>3</v>
       </c>
       <c r="I3" t="s">
+        <v>345</v>
+      </c>
+      <c r="J3" t="s">
         <v>346</v>
       </c>
-      <c r="J3" t="s">
-        <v>347</v>
-      </c>
       <c r="K3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
+        <v>347</v>
+      </c>
+      <c r="B4" t="s">
         <v>348</v>
       </c>
-      <c r="B4" t="s">
-        <v>349</v>
-      </c>
       <c r="C4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D4">
         <v>500</v>
@@ -5571,21 +5563,21 @@
         <v>3</v>
       </c>
       <c r="I4" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="J4" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="K4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
+        <v>353</v>
+      </c>
+      <c r="B5" t="s">
         <v>354</v>
-      </c>
-      <c r="B5" t="s">
-        <v>355</v>
       </c>
       <c r="D5">
         <v>500</v>
@@ -5594,33 +5586,33 @@
         <v>450</v>
       </c>
       <c r="F5" t="s">
+        <v>355</v>
+      </c>
+      <c r="G5" t="s">
         <v>356</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>357</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>358</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>359</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>360</v>
-      </c>
-      <c r="K5" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
+        <v>361</v>
+      </c>
+      <c r="B6" t="s">
         <v>362</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>363</v>
-      </c>
-      <c r="C6" t="s">
-        <v>364</v>
       </c>
       <c r="D6">
         <v>500</v>
@@ -5649,13 +5641,13 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
+        <v>361</v>
+      </c>
+      <c r="B7" t="s">
         <v>362</v>
       </c>
-      <c r="B7" t="s">
-        <v>363</v>
-      </c>
       <c r="C7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D7">
         <v>500</v>
@@ -5673,21 +5665,21 @@
         <v>3</v>
       </c>
       <c r="I7" t="s">
+        <v>364</v>
+      </c>
+      <c r="J7" t="s">
         <v>365</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>366</v>
-      </c>
-      <c r="K7" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
+        <v>367</v>
+      </c>
+      <c r="B8" t="s">
         <v>368</v>
-      </c>
-      <c r="B8" t="s">
-        <v>369</v>
       </c>
       <c r="D8">
         <v>500</v>
@@ -5716,10 +5708,10 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
+        <v>369</v>
+      </c>
+      <c r="B9" t="s">
         <v>370</v>
-      </c>
-      <c r="B9" t="s">
-        <v>371</v>
       </c>
       <c r="D9">
         <v>500</v>
@@ -5748,13 +5740,13 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
+        <v>371</v>
+      </c>
+      <c r="B10" t="s">
         <v>372</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>373</v>
-      </c>
-      <c r="C10" t="s">
-        <v>374</v>
       </c>
       <c r="D10">
         <v>500</v>
@@ -5763,33 +5755,33 @@
         <v>450</v>
       </c>
       <c r="F10" t="s">
+        <v>355</v>
+      </c>
+      <c r="G10" t="s">
         <v>356</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>357</v>
       </c>
-      <c r="H10" t="s">
-        <v>358</v>
-      </c>
       <c r="I10" t="s">
+        <v>345</v>
+      </c>
+      <c r="J10" t="s">
         <v>346</v>
       </c>
-      <c r="J10" t="s">
-        <v>347</v>
-      </c>
       <c r="K10" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
+        <v>371</v>
+      </c>
+      <c r="B11" t="s">
         <v>372</v>
       </c>
-      <c r="B11" t="s">
-        <v>373</v>
-      </c>
       <c r="C11" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D11">
         <v>500</v>
@@ -5798,13 +5790,13 @@
         <v>450</v>
       </c>
       <c r="F11" t="s">
+        <v>355</v>
+      </c>
+      <c r="G11" t="s">
         <v>356</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>357</v>
-      </c>
-      <c r="H11" t="s">
-        <v>358</v>
       </c>
       <c r="I11">
         <v>5</v>
@@ -5818,13 +5810,13 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
+        <v>371</v>
+      </c>
+      <c r="B12" t="s">
         <v>372</v>
       </c>
-      <c r="B12" t="s">
-        <v>373</v>
-      </c>
       <c r="C12" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D12">
         <v>500</v>
@@ -5833,13 +5825,13 @@
         <v>450</v>
       </c>
       <c r="F12" t="s">
+        <v>355</v>
+      </c>
+      <c r="G12" t="s">
         <v>356</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>357</v>
-      </c>
-      <c r="H12" t="s">
-        <v>358</v>
       </c>
       <c r="I12">
         <v>6</v>
@@ -5853,13 +5845,13 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
+        <v>371</v>
+      </c>
+      <c r="B13" t="s">
         <v>372</v>
       </c>
-      <c r="B13" t="s">
-        <v>373</v>
-      </c>
       <c r="C13" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D13">
         <v>500</v>
@@ -5868,13 +5860,13 @@
         <v>450</v>
       </c>
       <c r="F13" t="s">
+        <v>355</v>
+      </c>
+      <c r="G13" t="s">
         <v>356</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>357</v>
-      </c>
-      <c r="H13" t="s">
-        <v>358</v>
       </c>
       <c r="I13">
         <v>5</v>
@@ -5888,13 +5880,13 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
+        <v>376</v>
+      </c>
+      <c r="B14" t="s">
         <v>377</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>378</v>
-      </c>
-      <c r="C14" t="s">
-        <v>379</v>
       </c>
       <c r="D14">
         <v>500</v>
@@ -5903,33 +5895,33 @@
         <v>450</v>
       </c>
       <c r="F14" t="s">
+        <v>355</v>
+      </c>
+      <c r="G14" t="s">
         <v>356</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>357</v>
       </c>
-      <c r="H14" t="s">
-        <v>358</v>
-      </c>
       <c r="I14" t="s">
+        <v>345</v>
+      </c>
+      <c r="J14" t="s">
         <v>346</v>
       </c>
-      <c r="J14" t="s">
-        <v>347</v>
-      </c>
       <c r="K14" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
+        <v>376</v>
+      </c>
+      <c r="B15" t="s">
         <v>377</v>
       </c>
-      <c r="B15" t="s">
-        <v>378</v>
-      </c>
       <c r="C15" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D15">
         <v>500</v>
@@ -5938,13 +5930,13 @@
         <v>450</v>
       </c>
       <c r="F15" t="s">
+        <v>355</v>
+      </c>
+      <c r="G15" t="s">
         <v>356</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>357</v>
-      </c>
-      <c r="H15" t="s">
-        <v>358</v>
       </c>
       <c r="I15">
         <v>5</v>
@@ -5958,13 +5950,13 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
+        <v>376</v>
+      </c>
+      <c r="B16" t="s">
         <v>377</v>
       </c>
-      <c r="B16" t="s">
-        <v>378</v>
-      </c>
       <c r="C16" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D16">
         <v>500</v>
@@ -5973,13 +5965,13 @@
         <v>450</v>
       </c>
       <c r="F16" t="s">
+        <v>355</v>
+      </c>
+      <c r="G16" t="s">
         <v>356</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>357</v>
-      </c>
-      <c r="H16" t="s">
-        <v>358</v>
       </c>
       <c r="I16">
         <v>6</v>
@@ -5993,13 +5985,13 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
+        <v>376</v>
+      </c>
+      <c r="B17" t="s">
         <v>377</v>
       </c>
-      <c r="B17" t="s">
-        <v>378</v>
-      </c>
       <c r="C17" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D17">
         <v>500</v>
@@ -6008,13 +6000,13 @@
         <v>450</v>
       </c>
       <c r="F17" t="s">
+        <v>355</v>
+      </c>
+      <c r="G17" t="s">
         <v>356</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>357</v>
-      </c>
-      <c r="H17" t="s">
-        <v>358</v>
       </c>
       <c r="I17">
         <v>5</v>
@@ -6028,10 +6020,10 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
+        <v>379</v>
+      </c>
+      <c r="B18" t="s">
         <v>380</v>
-      </c>
-      <c r="B18" t="s">
-        <v>381</v>
       </c>
       <c r="D18">
         <v>500</v>
@@ -6060,10 +6052,10 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
+        <v>381</v>
+      </c>
+      <c r="B19" t="s">
         <v>382</v>
-      </c>
-      <c r="B19" t="s">
-        <v>383</v>
       </c>
       <c r="D19">
         <v>500</v>
@@ -6081,21 +6073,21 @@
         <v>3</v>
       </c>
       <c r="I19" t="s">
+        <v>383</v>
+      </c>
+      <c r="J19" t="s">
         <v>384</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>385</v>
-      </c>
-      <c r="K19" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
+        <v>386</v>
+      </c>
+      <c r="B20" t="s">
         <v>387</v>
-      </c>
-      <c r="B20" t="s">
-        <v>388</v>
       </c>
       <c r="D20">
         <v>500</v>
@@ -6113,21 +6105,21 @@
         <v>3</v>
       </c>
       <c r="I20" t="s">
+        <v>383</v>
+      </c>
+      <c r="J20" t="s">
         <v>384</v>
       </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>385</v>
-      </c>
-      <c r="K20" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
+        <v>388</v>
+      </c>
+      <c r="B21" t="s">
         <v>389</v>
-      </c>
-      <c r="B21" t="s">
-        <v>390</v>
       </c>
       <c r="D21">
         <v>500</v>
@@ -6156,10 +6148,10 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
+        <v>390</v>
+      </c>
+      <c r="B22" t="s">
         <v>391</v>
-      </c>
-      <c r="B22" t="s">
-        <v>392</v>
       </c>
       <c r="D22">
         <v>500</v>
@@ -6188,13 +6180,13 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
+        <v>392</v>
+      </c>
+      <c r="B23" t="s">
         <v>393</v>
       </c>
-      <c r="B23" t="s">
-        <v>394</v>
-      </c>
       <c r="C23" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D23">
         <v>500</v>
@@ -6223,13 +6215,13 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
+        <v>392</v>
+      </c>
+      <c r="B24" t="s">
         <v>393</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>394</v>
-      </c>
-      <c r="C24" t="s">
-        <v>395</v>
       </c>
       <c r="D24">
         <v>500</v>
@@ -6238,33 +6230,33 @@
         <v>450</v>
       </c>
       <c r="F24" t="s">
+        <v>344</v>
+      </c>
+      <c r="G24" t="s">
         <v>345</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>346</v>
       </c>
-      <c r="H24" t="s">
-        <v>347</v>
-      </c>
       <c r="I24" t="s">
+        <v>395</v>
+      </c>
+      <c r="J24" t="s">
         <v>396</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>397</v>
-      </c>
-      <c r="K24" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
+        <v>392</v>
+      </c>
+      <c r="B25" t="s">
         <v>393</v>
       </c>
-      <c r="B25" t="s">
-        <v>394</v>
-      </c>
       <c r="C25" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D25">
         <v>500</v>
@@ -6293,13 +6285,13 @@
     </row>
     <row r="26" spans="1:11">
       <c r="A26" t="s">
+        <v>398</v>
+      </c>
+      <c r="B26" t="s">
         <v>399</v>
       </c>
-      <c r="B26" t="s">
-        <v>400</v>
-      </c>
       <c r="C26" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D26">
         <v>500</v>
@@ -6308,33 +6300,33 @@
         <v>450</v>
       </c>
       <c r="F26" t="s">
+        <v>344</v>
+      </c>
+      <c r="G26" t="s">
         <v>345</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>346</v>
       </c>
-      <c r="H26" t="s">
-        <v>347</v>
-      </c>
       <c r="I26" t="s">
+        <v>395</v>
+      </c>
+      <c r="J26" t="s">
         <v>396</v>
       </c>
-      <c r="J26" t="s">
+      <c r="K26" t="s">
         <v>397</v>
-      </c>
-      <c r="K26" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
+        <v>398</v>
+      </c>
+      <c r="B27" t="s">
         <v>399</v>
       </c>
-      <c r="B27" t="s">
-        <v>400</v>
-      </c>
       <c r="C27" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D27">
         <v>500</v>
@@ -6363,13 +6355,13 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
+        <v>400</v>
+      </c>
+      <c r="B28" t="s">
         <v>401</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>402</v>
-      </c>
-      <c r="C28" t="s">
-        <v>403</v>
       </c>
       <c r="D28">
         <v>500</v>
@@ -6398,13 +6390,13 @@
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
+        <v>403</v>
+      </c>
+      <c r="B29" t="s">
         <v>404</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>405</v>
-      </c>
-      <c r="C29" t="s">
-        <v>406</v>
       </c>
       <c r="D29">
         <v>500</v>
@@ -6433,13 +6425,13 @@
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
+        <v>403</v>
+      </c>
+      <c r="B30" t="s">
         <v>404</v>
       </c>
-      <c r="B30" t="s">
-        <v>405</v>
-      </c>
       <c r="C30" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D30">
         <v>500</v>
@@ -6468,13 +6460,13 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
+        <v>406</v>
+      </c>
+      <c r="B31" t="s">
         <v>407</v>
       </c>
-      <c r="B31" t="s">
-        <v>408</v>
-      </c>
       <c r="C31" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D31">
         <v>500</v>
@@ -6503,13 +6495,13 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
+        <v>406</v>
+      </c>
+      <c r="B32" t="s">
         <v>407</v>
       </c>
-      <c r="B32" t="s">
-        <v>408</v>
-      </c>
       <c r="C32" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D32">
         <v>500</v>
@@ -6538,13 +6530,13 @@
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
+        <v>408</v>
+      </c>
+      <c r="B33" t="s">
         <v>409</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>410</v>
-      </c>
-      <c r="C33" t="s">
-        <v>411</v>
       </c>
       <c r="D33">
         <v>500</v>
@@ -6573,13 +6565,13 @@
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
+        <v>408</v>
+      </c>
+      <c r="B34" t="s">
         <v>409</v>
       </c>
-      <c r="B34" t="s">
-        <v>410</v>
-      </c>
       <c r="C34" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D34">
         <v>500</v>
@@ -6608,10 +6600,10 @@
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
+        <v>412</v>
+      </c>
+      <c r="B35" t="s">
         <v>413</v>
-      </c>
-      <c r="B35" t="s">
-        <v>414</v>
       </c>
       <c r="D35">
         <v>700</v>
@@ -6640,10 +6632,10 @@
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
+        <v>414</v>
+      </c>
+      <c r="B36" t="s">
         <v>415</v>
-      </c>
-      <c r="B36" t="s">
-        <v>416</v>
       </c>
       <c r="D36">
         <v>700</v>
@@ -6672,10 +6664,10 @@
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
+        <v>416</v>
+      </c>
+      <c r="B37" t="s">
         <v>417</v>
-      </c>
-      <c r="B37" t="s">
-        <v>418</v>
       </c>
       <c r="D37">
         <v>700</v>
@@ -6704,10 +6696,10 @@
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
+        <v>418</v>
+      </c>
+      <c r="B38" t="s">
         <v>419</v>
-      </c>
-      <c r="B38" t="s">
-        <v>420</v>
       </c>
       <c r="D38">
         <v>700</v>
@@ -6746,30 +6738,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>420</v>
+      </c>
+      <c r="B1" t="s">
         <v>421</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>422</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>423</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>424</v>
-      </c>
-      <c r="E1" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
+        <v>347</v>
+      </c>
+      <c r="B2" t="s">
         <v>348</v>
       </c>
-      <c r="B2" t="s">
-        <v>349</v>
-      </c>
       <c r="C2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
@@ -6780,13 +6772,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>353</v>
+      </c>
+      <c r="B3" t="s">
         <v>354</v>
       </c>
-      <c r="B3" t="s">
-        <v>355</v>
-      </c>
       <c r="C3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D3" t="b">
         <v>0</v>
@@ -6797,13 +6789,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
+        <v>371</v>
+      </c>
+      <c r="B4" t="s">
         <v>372</v>
       </c>
-      <c r="B4" t="s">
-        <v>373</v>
-      </c>
       <c r="C4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
@@ -6814,13 +6806,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B5" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -6831,13 +6823,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
+        <v>361</v>
+      </c>
+      <c r="B6" t="s">
         <v>362</v>
       </c>
-      <c r="B6" t="s">
-        <v>363</v>
-      </c>
       <c r="C6" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -6848,13 +6840,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
+        <v>367</v>
+      </c>
+      <c r="B7" t="s">
         <v>368</v>
       </c>
-      <c r="B7" t="s">
-        <v>369</v>
-      </c>
       <c r="C7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -6865,13 +6857,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
+        <v>369</v>
+      </c>
+      <c r="B8" t="s">
         <v>370</v>
       </c>
-      <c r="B8" t="s">
-        <v>371</v>
-      </c>
       <c r="C8" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
@@ -6882,13 +6874,13 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
+        <v>392</v>
+      </c>
+      <c r="B9" t="s">
         <v>393</v>
       </c>
-      <c r="B9" t="s">
-        <v>394</v>
-      </c>
       <c r="C9" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D9" t="b">
         <v>0</v>
@@ -6899,13 +6891,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
+        <v>408</v>
+      </c>
+      <c r="B10" t="s">
         <v>409</v>
       </c>
-      <c r="B10" t="s">
-        <v>410</v>
-      </c>
       <c r="C10" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D10" t="b">
         <v>0</v>
@@ -6916,13 +6908,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
+        <v>398</v>
+      </c>
+      <c r="B11" t="s">
         <v>399</v>
       </c>
-      <c r="B11" t="s">
-        <v>400</v>
-      </c>
       <c r="C11" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D11" t="b">
         <v>0</v>
@@ -6933,13 +6925,13 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
+        <v>400</v>
+      </c>
+      <c r="B12" t="s">
         <v>401</v>
       </c>
-      <c r="B12" t="s">
-        <v>402</v>
-      </c>
       <c r="C12" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D12" t="b">
         <v>0</v>
@@ -6950,13 +6942,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
+        <v>412</v>
+      </c>
+      <c r="B13" t="s">
         <v>413</v>
       </c>
-      <c r="B13" t="s">
-        <v>414</v>
-      </c>
       <c r="C13" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D13" t="b">
         <v>0</v>
@@ -6967,13 +6959,13 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
+        <v>414</v>
+      </c>
+      <c r="B14" t="s">
         <v>415</v>
       </c>
-      <c r="B14" t="s">
-        <v>416</v>
-      </c>
       <c r="C14" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D14" t="b">
         <v>0</v>
@@ -6984,13 +6976,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
+        <v>418</v>
+      </c>
+      <c r="B15" t="s">
         <v>419</v>
       </c>
-      <c r="B15" t="s">
-        <v>420</v>
-      </c>
       <c r="C15" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D15" t="b">
         <v>0</v>
@@ -7001,13 +6993,13 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
+        <v>416</v>
+      </c>
+      <c r="B16" t="s">
         <v>417</v>
       </c>
-      <c r="B16" t="s">
-        <v>418</v>
-      </c>
       <c r="C16" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D16" t="b">
         <v>0</v>
@@ -7018,13 +7010,13 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
+        <v>403</v>
+      </c>
+      <c r="B17" t="s">
         <v>404</v>
       </c>
-      <c r="B17" t="s">
-        <v>405</v>
-      </c>
       <c r="C17" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D17" t="b">
         <v>0</v>
@@ -7035,13 +7027,13 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B18" t="s">
         <v>407</v>
       </c>
-      <c r="B18" t="s">
-        <v>408</v>
-      </c>
       <c r="C18" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D18" t="b">
         <v>0</v>
@@ -7052,13 +7044,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
+        <v>381</v>
+      </c>
+      <c r="B19" t="s">
         <v>382</v>
       </c>
-      <c r="B19" t="s">
-        <v>383</v>
-      </c>
       <c r="C19" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D19" t="b">
         <v>0</v>
@@ -7069,13 +7061,13 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
+        <v>386</v>
+      </c>
+      <c r="B20" t="s">
         <v>387</v>
       </c>
-      <c r="B20" t="s">
-        <v>388</v>
-      </c>
       <c r="C20" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D20" t="b">
         <v>0</v>
@@ -7086,13 +7078,13 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
+        <v>390</v>
+      </c>
+      <c r="B21" t="s">
         <v>391</v>
       </c>
-      <c r="B21" t="s">
-        <v>392</v>
-      </c>
       <c r="C21" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D21" t="b">
         <v>0</v>
@@ -7103,13 +7095,13 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
+        <v>388</v>
+      </c>
+      <c r="B22" t="s">
         <v>389</v>
       </c>
-      <c r="B22" t="s">
-        <v>390</v>
-      </c>
       <c r="C22" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D22" t="b">
         <v>0</v>
@@ -7120,13 +7112,13 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
+        <v>379</v>
+      </c>
+      <c r="B23" t="s">
         <v>380</v>
       </c>
-      <c r="B23" t="s">
-        <v>381</v>
-      </c>
       <c r="C23" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D23" t="b">
         <v>0</v>
@@ -7147,21 +7139,21 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B1" t="s">
         <v>430</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>431</v>
-      </c>
-      <c r="C1" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B2" t="s">
         <v>433</v>
-      </c>
-      <c r="B2" t="s">
-        <v>434</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -7169,10 +7161,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -7180,10 +7172,10 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B4" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -7191,10 +7183,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B5" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C5">
         <v>3</v>
@@ -7202,10 +7194,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B6" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -7213,10 +7205,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B7" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -7224,10 +7216,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B8" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -7235,10 +7227,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B9" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -7246,10 +7238,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B10" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -7257,10 +7249,10 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B11" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -7268,10 +7260,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B12" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -7279,10 +7271,10 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B13" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -7290,10 +7282,10 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B14" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C14">
         <v>3</v>
@@ -7301,10 +7293,10 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B15" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -7312,10 +7304,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B16" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -7323,10 +7315,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B17" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C17">
         <v>3</v>
@@ -7334,10 +7326,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B18" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -7345,10 +7337,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B19" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -7356,10 +7348,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B20" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -7367,10 +7359,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -7378,10 +7370,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B22" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C22">
         <v>2</v>
@@ -7389,10 +7381,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B23" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -7400,10 +7392,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B24" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -7411,10 +7403,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B25" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C25">
         <v>3</v>
@@ -7422,10 +7414,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B26" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C26">
         <v>3</v>
@@ -7433,10 +7425,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B27" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C27">
         <v>2</v>
@@ -7444,10 +7436,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B28" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C28">
         <v>3</v>
@@ -7455,10 +7447,10 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B29" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -7466,10 +7458,10 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B30" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -7477,10 +7469,10 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B31" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -7488,10 +7480,10 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B32" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -7499,10 +7491,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B33" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -7510,10 +7502,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B34" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -7521,10 +7513,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B35" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C35">
         <v>2</v>
@@ -7532,10 +7524,10 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B36" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -7543,10 +7535,10 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B37" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C37">
         <v>3</v>
@@ -7564,16 +7556,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
+        <v>445</v>
+      </c>
+      <c r="B1" t="s">
         <v>446</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>447</v>
       </c>
-      <c r="C1" t="s">
-        <v>448</v>
-      </c>
       <c r="D1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -7587,7 +7579,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -7601,7 +7593,7 @@
         <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -7615,7 +7607,7 @@
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -7629,7 +7621,7 @@
         <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -7643,7 +7635,7 @@
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -7657,7 +7649,7 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -7671,7 +7663,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -7685,7 +7677,7 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -7699,7 +7691,7 @@
         <v>38</v>
       </c>
       <c r="D10" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -7713,7 +7705,7 @@
         <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -7727,7 +7719,7 @@
         <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -7741,7 +7733,7 @@
         <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -7755,7 +7747,7 @@
         <v>6</v>
       </c>
       <c r="D14" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -7769,7 +7761,7 @@
         <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -7783,7 +7775,7 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -7797,7 +7789,7 @@
         <v>6</v>
       </c>
       <c r="D17" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -7811,7 +7803,7 @@
         <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -7825,7 +7817,7 @@
         <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -7839,7 +7831,7 @@
         <v>38</v>
       </c>
       <c r="D20" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -7853,7 +7845,7 @@
         <v>38</v>
       </c>
       <c r="D21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -7867,7 +7859,7 @@
         <v>6</v>
       </c>
       <c r="D22" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -7881,7 +7873,7 @@
         <v>6</v>
       </c>
       <c r="D23" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -7895,7 +7887,7 @@
         <v>6</v>
       </c>
       <c r="D24" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -7909,7 +7901,7 @@
         <v>38</v>
       </c>
       <c r="D25" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -7923,7 +7915,7 @@
         <v>38</v>
       </c>
       <c r="D26" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -7937,7 +7929,7 @@
         <v>38</v>
       </c>
       <c r="D27" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -7951,7 +7943,7 @@
         <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -7965,7 +7957,7 @@
         <v>6</v>
       </c>
       <c r="D29" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -7979,7 +7971,7 @@
         <v>38</v>
       </c>
       <c r="D30" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -7993,7 +7985,7 @@
         <v>38</v>
       </c>
       <c r="D31" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -8007,7 +7999,7 @@
         <v>38</v>
       </c>
       <c r="D32" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>